<commit_message>
Updated IND_grids_kan10 model - 2026-08-31 16:50
</commit_message>
<xml_diff>
--- a/VerveStacks_IND_grids_kan10/Sets-vervestacks.xlsx
+++ b/VerveStacks_IND_grids_kan10/Sets-vervestacks.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\VEDA\Veda\Veda_models\vervestacks_models\VerveStacks_IND_grids_kan10\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{67BE9650-0457-4EBC-9BEC-CC4D74BDAD2F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9BCF3DA7-C385-4196-88F5-D97CEC27D7DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="390" yWindow="390" windowWidth="21600" windowHeight="11295" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1950" yWindow="1950" windowWidth="21600" windowHeight="11295" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="VEDA_Sets-Comm" sheetId="2" r:id="rId1"/>
@@ -2319,7 +2319,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DB36B221-3A0E-4728-A9AC-E0EDFE254361}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0CDD270A-1AAB-497F-BC84-40381B8BE005}">
   <dimension ref="B9:E195"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated IND_grids_kan10 model - 2026-08-31 17:57
</commit_message>
<xml_diff>
--- a/VerveStacks_IND_grids_kan10/Sets-vervestacks.xlsx
+++ b/VerveStacks_IND_grids_kan10/Sets-vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\VEDA\Veda\Veda_models\vervestacks_models\VerveStacks_IND_grids_kan10\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC68658F-DA51-4DF0-96B4-B0D52C1F77CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B7E14EC-CDC9-46D4-9FE9-0FB04C1E9DBF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1950" yWindow="1950" windowWidth="21600" windowHeight="11295" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="868" uniqueCount="479">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="864" uniqueCount="477">
   <si>
     <t>~TFM_Psets</t>
   </si>
@@ -1325,12 +1325,6 @@
   </si>
   <si>
     <t>elc_won_IND_066</t>
-  </si>
-  <si>
-    <t>rez_won_IND_067</t>
-  </si>
-  <si>
-    <t>elc_won_IND_067</t>
   </si>
   <si>
     <t>rez_wof_IND_001</t>
@@ -2319,8 +2313,8 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{369486DE-D244-4264-95D3-872289C16F30}">
-  <dimension ref="B9:E195"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B6BAAC29-BAE0-4259-80EC-FAD5FF74EC9E}">
+  <dimension ref="B9:E194"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="9" spans="2:5" x14ac:dyDescent="0.25">
@@ -4915,20 +4909,6 @@
         <v>476</v>
       </c>
       <c r="E194" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="195" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B195" t="s">
-        <v>477</v>
-      </c>
-      <c r="C195" t="s">
-        <v>478</v>
-      </c>
-      <c r="D195" t="s">
-        <v>478</v>
-      </c>
-      <c r="E195" t="s">
         <v>110</v>
       </c>
     </row>

</xml_diff>